<commit_message>
Show TRM's chosen comparable projects, and why, on each project's Investor tab
scripts/data/comparables-from-sheet.py reads the comparables TRM chose in
the project sheet (50 of the 97 map projects), locates each on OneMap
(address, district, distance, under construction) and matches it to the
Huttons catalogue (tenure, units, completion). chosen-notes.ts explains each
choice in plain words from TRM's note, with figures only from the note
(credited to TRM), OneMap or the catalogue; tests check the distances.

Each chosen project's Investor tab (and coming-soon page) shows the
comparable, why it's comparable, the facts side by side, a warning where the
comparable is still being built, and that its URA resale and rental records
are still to be loaded. TRM's entries are carried into the 97-project sheet.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KW7zaXcExZeiPiJSUazWYH
</commit_message>
<xml_diff>
--- a/exports/trm-map-projects-comparables.xlsx
+++ b/exports/trm-map-projects-comparables.xlsx
@@ -487,7 +487,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q104"/>
+  <dimension ref="A1:Q103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -811,8 +811,16 @@
           <t>00a420908c8249778e11c7d2259afb18</t>
         </is>
       </c>
-      <c r="O8" s="9" t="n"/>
-      <c r="P8" s="9" t="n"/>
+      <c r="O8" s="9" t="inlineStr">
+        <is>
+          <t>THE LINQ @ BEAUTY WORLD</t>
+        </is>
+      </c>
+      <c r="P8" s="9" t="inlineStr">
+        <is>
+          <t>Similar number of units, projects right next to each other</t>
+        </is>
+      </c>
       <c r="Q8" s="10" t="n"/>
     </row>
     <row r="9">
@@ -1018,8 +1026,16 @@
           <t>f8b877eb3d354bdfa56ef5b1b60924ca</t>
         </is>
       </c>
-      <c r="O11" s="9" t="n"/>
-      <c r="P11" s="9" t="n"/>
+      <c r="O11" s="9" t="inlineStr">
+        <is>
+          <t>ONE MEYER</t>
+        </is>
+      </c>
+      <c r="P11" s="9" t="inlineStr">
+        <is>
+          <t>Most recent new launch and similar location, but has 10 profitable : 1 unprofitable</t>
+        </is>
+      </c>
       <c r="Q11" s="10" t="n"/>
     </row>
     <row r="12">
@@ -1295,8 +1311,16 @@
           <t>d628a74456874b778432799fd9e53517</t>
         </is>
       </c>
-      <c r="O15" s="9" t="n"/>
-      <c r="P15" s="9" t="n"/>
+      <c r="O15" s="9" t="inlineStr">
+        <is>
+          <t>SCENECA RESIDENCE</t>
+        </is>
+      </c>
+      <c r="P15" s="9" t="inlineStr">
+        <is>
+          <t>Sceneca is the closest new launch in scale and profitability</t>
+        </is>
+      </c>
       <c r="Q15" s="10" t="n"/>
     </row>
     <row r="16">
@@ -1362,8 +1386,16 @@
           <t>0855eefe285a456783eeda789a0203cf</t>
         </is>
       </c>
-      <c r="O16" s="9" t="n"/>
-      <c r="P16" s="9" t="n"/>
+      <c r="O16" s="9" t="inlineStr">
+        <is>
+          <t>SCENECA RESIDENCE</t>
+        </is>
+      </c>
+      <c r="P16" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Similar number of units, both nearby Tanah Merah MRT </t>
+        </is>
+      </c>
       <c r="Q16" s="10" t="n"/>
     </row>
     <row r="17">
@@ -1500,8 +1532,16 @@
           <t>2546baa1d7364ff1b2024aa98c49a248</t>
         </is>
       </c>
-      <c r="O18" s="9" t="n"/>
-      <c r="P18" s="9" t="n"/>
+      <c r="O18" s="9" t="inlineStr">
+        <is>
+          <t>COMMONWEALTH TOWERS</t>
+        </is>
+      </c>
+      <c r="P18" s="9" t="inlineStr">
+        <is>
+          <t>Closest recent new launch in terms of location and size</t>
+        </is>
+      </c>
       <c r="Q18" s="10" t="n"/>
     </row>
     <row r="19">
@@ -1569,8 +1609,16 @@
           <t>697564dce09a4511a8d56e739ecdaabd</t>
         </is>
       </c>
-      <c r="O19" s="9" t="n"/>
-      <c r="P19" s="9" t="n"/>
+      <c r="O19" s="9" t="inlineStr">
+        <is>
+          <t>WATERGARDENS @ CANBERRA</t>
+        </is>
+      </c>
+      <c r="P19" s="9" t="inlineStr">
+        <is>
+          <t>Similar location and scale</t>
+        </is>
+      </c>
       <c r="Q19" s="10" t="n"/>
     </row>
     <row r="20">
@@ -1638,8 +1686,16 @@
           <t>227b5a5863fa4631875adcfb07b38cae</t>
         </is>
       </c>
-      <c r="O20" s="9" t="n"/>
-      <c r="P20" s="9" t="n"/>
+      <c r="O20" s="9" t="inlineStr">
+        <is>
+          <t>THE IMPERIAL</t>
+        </is>
+      </c>
+      <c r="P20" s="9" t="inlineStr">
+        <is>
+          <t>Old condo (2006) but fully profitable at 100+ transactions</t>
+        </is>
+      </c>
       <c r="Q20" s="10" t="n"/>
     </row>
     <row r="21">
@@ -1844,8 +1900,16 @@
           <t>a8dc1c7b80914f65a5c07128aaa9e777</t>
         </is>
       </c>
-      <c r="O23" s="9" t="n"/>
-      <c r="P23" s="9" t="n"/>
+      <c r="O23" s="9" t="inlineStr">
+        <is>
+          <t>THE ESTUARY</t>
+        </is>
+      </c>
+      <c r="P23" s="9" t="inlineStr">
+        <is>
+          <t>Old condo (2008) but very nearby and fully profitable at 123 transactions</t>
+        </is>
+      </c>
       <c r="Q23" s="10" t="n"/>
     </row>
     <row r="24">
@@ -1913,8 +1977,16 @@
           <t>eccc7150c2254954a2371b9655eb459c</t>
         </is>
       </c>
-      <c r="O24" s="9" t="n"/>
-      <c r="P24" s="9" t="n"/>
+      <c r="O24" s="9" t="inlineStr">
+        <is>
+          <t>THE SCALA</t>
+        </is>
+      </c>
+      <c r="P24" s="9" t="inlineStr">
+        <is>
+          <t>Quite an old condo (2013) but fully profitable and the newest in the area</t>
+        </is>
+      </c>
       <c r="Q24" s="10" t="n"/>
     </row>
     <row r="25">
@@ -2049,8 +2121,16 @@
           <t>679021ecbcab48be90b64e16e77b82b7</t>
         </is>
       </c>
-      <c r="O26" s="9" t="n"/>
-      <c r="P26" s="9" t="n"/>
+      <c r="O26" s="9" t="inlineStr">
+        <is>
+          <t>TWIN FOUNTAINS</t>
+        </is>
+      </c>
+      <c r="P26" s="9" t="inlineStr">
+        <is>
+          <t>Close to Clovelle of Woodlands and fully profitable at 179 transactions</t>
+        </is>
+      </c>
       <c r="Q26" s="10" t="n"/>
     </row>
     <row r="27">
@@ -2118,8 +2198,16 @@
           <t>60dab94999134e819496275b30b239aa</t>
         </is>
       </c>
-      <c r="O27" s="9" t="n"/>
-      <c r="P27" s="9" t="n"/>
+      <c r="O27" s="9" t="inlineStr">
+        <is>
+          <t>PASIR RIS 8 or RIPPLE BAY</t>
+        </is>
+      </c>
+      <c r="P27" s="9" t="inlineStr">
+        <is>
+          <t>Pasir Ris 8 - Most recent new launch Ripple Bay - Closer in terms of similar location</t>
+        </is>
+      </c>
       <c r="Q27" s="10" t="n"/>
     </row>
     <row r="28">
@@ -2323,8 +2411,16 @@
           <t>cf6fa6bd96944f56ae7ea4d8bdb162cd</t>
         </is>
       </c>
-      <c r="O30" s="9" t="n"/>
-      <c r="P30" s="9" t="n"/>
+      <c r="O30" s="9" t="inlineStr">
+        <is>
+          <t>DAIRY FARM RESIDENCES</t>
+        </is>
+      </c>
+      <c r="P30" s="9" t="inlineStr">
+        <is>
+          <t>Similar location, profitable ot unprofitable 67:3</t>
+        </is>
+      </c>
       <c r="Q30" s="10" t="n"/>
     </row>
     <row r="31">
@@ -2531,8 +2627,16 @@
           <t>88a853a0ae6443749b7e5f957b8e6480</t>
         </is>
       </c>
-      <c r="O33" s="9" t="n"/>
-      <c r="P33" s="9" t="n"/>
+      <c r="O33" s="9" t="inlineStr">
+        <is>
+          <t>THE CLEMENT CANOPY</t>
+        </is>
+      </c>
+      <c r="P33" s="9" t="inlineStr">
+        <is>
+          <t>Same district and similar area with similar scale, full positive transactions</t>
+        </is>
+      </c>
       <c r="Q33" s="10" t="n"/>
     </row>
     <row r="34">
@@ -2600,8 +2704,16 @@
           <t>946c32a7bc3c43f6b1df4513a33d371e</t>
         </is>
       </c>
-      <c r="O34" s="9" t="n"/>
-      <c r="P34" s="9" t="n"/>
+      <c r="O34" s="9" t="inlineStr">
+        <is>
+          <t>THE CLEMENT CANOPY</t>
+        </is>
+      </c>
+      <c r="P34" s="9" t="inlineStr">
+        <is>
+          <t>Same district and similar area with similar scale, full positive transactions</t>
+        </is>
+      </c>
       <c r="Q34" s="10" t="n"/>
     </row>
     <row r="35">
@@ -2669,8 +2781,16 @@
           <t>3c4e53308b2c48d0bca49a3984e36eaa</t>
         </is>
       </c>
-      <c r="O35" s="9" t="n"/>
-      <c r="P35" s="9" t="n"/>
+      <c r="O35" s="9" t="inlineStr">
+        <is>
+          <t>THE RESERVE RESIDENCES</t>
+        </is>
+      </c>
+      <c r="P35" s="9" t="inlineStr">
+        <is>
+          <t>Similar area</t>
+        </is>
+      </c>
       <c r="Q35" s="10" t="n"/>
     </row>
     <row r="36">
@@ -2951,8 +3071,16 @@
           <t>1430cfcb8f9c4302860203c0f370a169</t>
         </is>
       </c>
-      <c r="O39" s="9" t="n"/>
-      <c r="P39" s="9" t="n"/>
+      <c r="O39" s="9" t="inlineStr">
+        <is>
+          <t>LIV @ MB</t>
+        </is>
+      </c>
+      <c r="P39" s="9" t="inlineStr">
+        <is>
+          <t>Fully profitable and similar location</t>
+        </is>
+      </c>
       <c r="Q39" s="10" t="n"/>
     </row>
     <row r="40">
@@ -3156,8 +3284,16 @@
           <t>7fc6731e8e4a4121a433521c68998c0c</t>
         </is>
       </c>
-      <c r="O42" s="9" t="n"/>
-      <c r="P42" s="9" t="n"/>
+      <c r="O42" s="9" t="inlineStr">
+        <is>
+          <t>RIVERFRONT RESIDENCES</t>
+        </is>
+      </c>
+      <c r="P42" s="9" t="inlineStr">
+        <is>
+          <t>Fully profitable at 500+ transactions, in Hougang area too</t>
+        </is>
+      </c>
       <c r="Q42" s="10" t="n"/>
     </row>
     <row r="43">
@@ -3225,8 +3361,16 @@
           <t>e80c8fc512304bd7b7969fcf96b00048</t>
         </is>
       </c>
-      <c r="O43" s="9" t="n"/>
-      <c r="P43" s="9" t="n"/>
+      <c r="O43" s="9" t="inlineStr">
+        <is>
+          <t>COMMONWEALTH TOWERS</t>
+        </is>
+      </c>
+      <c r="P43" s="9" t="inlineStr">
+        <is>
+          <t>Closest recent new launch in terms of location and size</t>
+        </is>
+      </c>
       <c r="Q43" s="10" t="n"/>
     </row>
     <row r="44">
@@ -3294,8 +3438,16 @@
           <t>b43a59ee25424f54adb7ea7639a7aee5</t>
         </is>
       </c>
-      <c r="O44" s="9" t="n"/>
-      <c r="P44" s="9" t="n"/>
+      <c r="O44" s="9" t="inlineStr">
+        <is>
+          <t>J Gateway</t>
+        </is>
+      </c>
+      <c r="P44" s="9" t="inlineStr">
+        <is>
+          <t>Similar location, 150:1 profitable to unprofitable</t>
+        </is>
+      </c>
       <c r="Q44" s="10" t="n"/>
     </row>
     <row r="45">
@@ -3432,8 +3584,16 @@
           <t>ad0b6595310b4a0e9bcf1811adab01d1</t>
         </is>
       </c>
-      <c r="O46" s="9" t="n"/>
-      <c r="P46" s="9" t="n"/>
+      <c r="O46" s="9" t="inlineStr">
+        <is>
+          <t>PARC KOMO</t>
+        </is>
+      </c>
+      <c r="P46" s="9" t="inlineStr">
+        <is>
+          <t>Similar location &amp; size, and fully profitable at 43 transactions</t>
+        </is>
+      </c>
       <c r="Q46" s="10" t="n"/>
     </row>
     <row r="47">
@@ -3639,8 +3799,16 @@
           <t>02a030d8f3ca4ed1b2093e94e3b31115</t>
         </is>
       </c>
-      <c r="O49" s="9" t="n"/>
-      <c r="P49" s="9" t="n"/>
+      <c r="O49" s="9" t="inlineStr">
+        <is>
+          <t>LENTOR MODERN</t>
+        </is>
+      </c>
+      <c r="P49" s="9" t="inlineStr">
+        <is>
+          <t>Same location, 61:1 profitable to unprofitable</t>
+        </is>
+      </c>
       <c r="Q49" s="10" t="n"/>
     </row>
     <row r="50">
@@ -3708,8 +3876,16 @@
           <t>e0d7efea415743a79d08cda8de572c09</t>
         </is>
       </c>
-      <c r="O50" s="9" t="n"/>
-      <c r="P50" s="9" t="n"/>
+      <c r="O50" s="9" t="inlineStr">
+        <is>
+          <t>LENTOR MODERN</t>
+        </is>
+      </c>
+      <c r="P50" s="9" t="inlineStr">
+        <is>
+          <t>Same location, 61:1 profitable to unprofitable</t>
+        </is>
+      </c>
       <c r="Q50" s="10" t="n"/>
     </row>
     <row r="51">
@@ -3777,8 +3953,16 @@
           <t>adf9b59f73ba40cc85938836a28d4037</t>
         </is>
       </c>
-      <c r="O51" s="9" t="n"/>
-      <c r="P51" s="9" t="n"/>
+      <c r="O51" s="9" t="inlineStr">
+        <is>
+          <t>LAKE GRANDE</t>
+        </is>
+      </c>
+      <c r="P51" s="9" t="inlineStr">
+        <is>
+          <t>Fully profitable and similar location with the same views</t>
+        </is>
+      </c>
       <c r="Q51" s="10" t="n"/>
     </row>
     <row r="52">
@@ -3846,8 +4030,16 @@
           <t>83b9b826f1f0445ca23b38813aea6358</t>
         </is>
       </c>
-      <c r="O52" s="9" t="n"/>
-      <c r="P52" s="9" t="n"/>
+      <c r="O52" s="9" t="inlineStr">
+        <is>
+          <t>AMBER PARK</t>
+        </is>
+      </c>
+      <c r="P52" s="9" t="inlineStr">
+        <is>
+          <t>Similar location, fully profitable at 87 transactions</t>
+        </is>
+      </c>
       <c r="Q52" s="10" t="n"/>
     </row>
     <row r="53">
@@ -3913,8 +4105,16 @@
           <t>b83a142f417049e58c49b5be22ab0cea</t>
         </is>
       </c>
-      <c r="O53" s="9" t="n"/>
-      <c r="P53" s="9" t="n"/>
+      <c r="O53" s="9" t="inlineStr">
+        <is>
+          <t>THE CRITERION</t>
+        </is>
+      </c>
+      <c r="P53" s="9" t="inlineStr">
+        <is>
+          <t>Similar location, and also fully profitable at 240+ transactions</t>
+        </is>
+      </c>
       <c r="Q53" s="10" t="n"/>
     </row>
     <row r="54">
@@ -3989,8 +4189,16 @@
           <t>030fee210b074a86a512f1f6cfaf62b6</t>
         </is>
       </c>
-      <c r="O54" s="9" t="n"/>
-      <c r="P54" s="9" t="n"/>
+      <c r="O54" s="9" t="inlineStr">
+        <is>
+          <t>THE RESERVE RESIDENCES</t>
+        </is>
+      </c>
+      <c r="P54" s="9" t="inlineStr">
+        <is>
+          <t>Similar location and scale</t>
+        </is>
+      </c>
       <c r="Q54" s="10" t="n"/>
     </row>
     <row r="55">
@@ -4059,8 +4267,16 @@
           <t>4a25b483869c44f38fad81c15c945c4f</t>
         </is>
       </c>
-      <c r="O55" s="9" t="n"/>
-      <c r="P55" s="9" t="n"/>
+      <c r="O55" s="9" t="inlineStr">
+        <is>
+          <t>THE RESERVE RESIDENCES</t>
+        </is>
+      </c>
+      <c r="P55" s="9" t="inlineStr">
+        <is>
+          <t>Similar location and scale</t>
+        </is>
+      </c>
       <c r="Q55" s="10" t="n"/>
     </row>
     <row r="56">
@@ -4197,8 +4413,16 @@
           <t>e2f59c122d1b47af8d9a734fc79fa467</t>
         </is>
       </c>
-      <c r="O57" s="9" t="n"/>
-      <c r="P57" s="9" t="n"/>
+      <c r="O57" s="9" t="inlineStr">
+        <is>
+          <t>SYMPHONY SUITES</t>
+        </is>
+      </c>
+      <c r="P57" s="9" t="inlineStr">
+        <is>
+          <t>Similar location, fully profitable at 244 transactions</t>
+        </is>
+      </c>
       <c r="Q57" s="10" t="n"/>
     </row>
     <row r="58">
@@ -4266,8 +4490,16 @@
           <t>3afb1fde3a244b79bc85e5f39d888ab4</t>
         </is>
       </c>
-      <c r="O58" s="9" t="n"/>
-      <c r="P58" s="9" t="n"/>
+      <c r="O58" s="9" t="inlineStr">
+        <is>
+          <t>PARC ROSEWOOD</t>
+        </is>
+      </c>
+      <c r="P58" s="9" t="inlineStr">
+        <is>
+          <t>Similar location, and best profit ratio at 210:5 profitable to unprofitable transactions</t>
+        </is>
+      </c>
       <c r="Q58" s="10" t="n"/>
     </row>
     <row r="59">
@@ -4402,8 +4634,16 @@
           <t>f12c41ea74b5463a91ff0c84f7481218</t>
         </is>
       </c>
-      <c r="O60" s="9" t="n"/>
-      <c r="P60" s="9" t="n"/>
+      <c r="O60" s="9" t="inlineStr">
+        <is>
+          <t>THE SCALA</t>
+        </is>
+      </c>
+      <c r="P60" s="9" t="inlineStr">
+        <is>
+          <t>Quite an old condo (2013) but fully profitable and the newest in the area</t>
+        </is>
+      </c>
       <c r="Q60" s="10" t="n"/>
     </row>
     <row r="61">
@@ -4472,8 +4712,16 @@
           <t>b1d78cceab4d4515a1ec7969ccda74b8</t>
         </is>
       </c>
-      <c r="O61" s="9" t="n"/>
-      <c r="P61" s="9" t="n"/>
+      <c r="O61" s="9" t="inlineStr">
+        <is>
+          <t>THE SAIL @ MARINA BAY</t>
+        </is>
+      </c>
+      <c r="P61" s="9" t="inlineStr">
+        <is>
+          <t>Similar location, best profit ratio nearby at 229:17 profitable to unprofitable</t>
+        </is>
+      </c>
       <c r="Q61" s="10" t="n"/>
     </row>
     <row r="62">
@@ -4612,8 +4860,16 @@
           <t>af5940a962684cb1ac366e1535d1b7a0</t>
         </is>
       </c>
-      <c r="O63" s="9" t="n"/>
-      <c r="P63" s="9" t="n"/>
+      <c r="O63" s="9" t="inlineStr">
+        <is>
+          <t>TREASURE AT TAMPINES</t>
+        </is>
+      </c>
+      <c r="P63" s="9" t="inlineStr">
+        <is>
+          <t>both mega developments, also at D18</t>
+        </is>
+      </c>
       <c r="Q63" s="10" t="n"/>
     </row>
     <row r="64">
@@ -4683,8 +4939,16 @@
           <t>31378b5622d24478bc68a07ddc399c65</t>
         </is>
       </c>
-      <c r="O64" s="9" t="n"/>
-      <c r="P64" s="9" t="n"/>
+      <c r="O64" s="9" t="inlineStr">
+        <is>
+          <t>STIRLING RESIDENCES</t>
+        </is>
+      </c>
+      <c r="P64" s="9" t="inlineStr">
+        <is>
+          <t>Extremely high profitability ratio</t>
+        </is>
+      </c>
       <c r="Q64" s="10" t="n"/>
     </row>
     <row r="65">
@@ -4752,8 +5016,16 @@
           <t>eaf892dde8d345e7b8beea79e9851184</t>
         </is>
       </c>
-      <c r="O65" s="9" t="n"/>
-      <c r="P65" s="9" t="n"/>
+      <c r="O65" s="9" t="inlineStr">
+        <is>
+          <t>PARC CENTRAL RESIDENCES</t>
+        </is>
+      </c>
+      <c r="P65" s="9" t="inlineStr">
+        <is>
+          <t>At Tampines West too, all profitable</t>
+        </is>
+      </c>
       <c r="Q65" s="10" t="n"/>
     </row>
     <row r="66">
@@ -4821,8 +5093,16 @@
           <t>1917872113dc425797ca4239311a6ee3</t>
         </is>
       </c>
-      <c r="O66" s="9" t="n"/>
-      <c r="P66" s="9" t="n"/>
+      <c r="O66" s="9" t="inlineStr">
+        <is>
+          <t>IRWELL HILL RESIDENCES</t>
+        </is>
+      </c>
+      <c r="P66" s="9" t="inlineStr">
+        <is>
+          <t>Similar location and new, good profitability ratio at 42:3 profitable to unprofitable</t>
+        </is>
+      </c>
       <c r="Q66" s="10" t="n"/>
     </row>
     <row r="67">
@@ -5026,8 +5306,16 @@
           <t>f62ad7ec239241fa8a8bd10dacaf8291</t>
         </is>
       </c>
-      <c r="O69" s="9" t="n"/>
-      <c r="P69" s="9" t="n"/>
+      <c r="O69" s="9" t="inlineStr">
+        <is>
+          <t>WATERGARDENS @ CANBERRA</t>
+        </is>
+      </c>
+      <c r="P69" s="9" t="inlineStr">
+        <is>
+          <t>Similar location and scale</t>
+        </is>
+      </c>
       <c r="Q69" s="10" t="n"/>
     </row>
     <row r="70">
@@ -5298,8 +5586,16 @@
           <t>478f87cc6ca64393bc3aea90f798f484</t>
         </is>
       </c>
-      <c r="O73" s="9" t="n"/>
-      <c r="P73" s="9" t="n"/>
+      <c r="O73" s="9" t="inlineStr">
+        <is>
+          <t>CHESTERVALE</t>
+        </is>
+      </c>
+      <c r="P73" s="9" t="inlineStr">
+        <is>
+          <t>Super old condo (1999) but was also an EC and fully profitable at 51 transactions.</t>
+        </is>
+      </c>
       <c r="Q73" s="10" t="n"/>
     </row>
     <row r="74">
@@ -5505,8 +5801,16 @@
           <t>5862d7b906c54440828e1269d19bf2fc</t>
         </is>
       </c>
-      <c r="O76" s="9" t="n"/>
-      <c r="P76" s="9" t="n"/>
+      <c r="O76" s="9" t="inlineStr">
+        <is>
+          <t>LAKE GRANDE</t>
+        </is>
+      </c>
+      <c r="P76" s="9" t="inlineStr">
+        <is>
+          <t>Similar location and views</t>
+        </is>
+      </c>
       <c r="Q76" s="10" t="n"/>
     </row>
     <row r="77">
@@ -5644,8 +5948,16 @@
           <t>997843e71ffa45d08e3f20e2a0fd96ed</t>
         </is>
       </c>
-      <c r="O78" s="9" t="n"/>
-      <c r="P78" s="9" t="n"/>
+      <c r="O78" s="9" t="inlineStr">
+        <is>
+          <t>LENTOR MODERN</t>
+        </is>
+      </c>
+      <c r="P78" s="9" t="inlineStr">
+        <is>
+          <t>Closeby in location, 61:1 profitable to unprofitable</t>
+        </is>
+      </c>
       <c r="Q78" s="10" t="n"/>
     </row>
     <row r="79">
@@ -5713,8 +6025,16 @@
           <t>655c7d587a7943a2b95bed4d0b4bf182</t>
         </is>
       </c>
-      <c r="O79" s="9" t="n"/>
-      <c r="P79" s="9" t="n"/>
+      <c r="O79" s="9" t="inlineStr">
+        <is>
+          <t>KENT RIDGE HILL RESIDENCES</t>
+        </is>
+      </c>
+      <c r="P79" s="9" t="inlineStr">
+        <is>
+          <t>Closeby in location, fully profitable at 106 transactions.</t>
+        </is>
+      </c>
       <c r="Q79" s="10" t="n"/>
     </row>
     <row r="80">
@@ -5782,8 +6102,16 @@
           <t>81f063c801ef487f8a695b825e20c30c</t>
         </is>
       </c>
-      <c r="O80" s="9" t="n"/>
-      <c r="P80" s="9" t="n"/>
+      <c r="O80" s="9" t="inlineStr">
+        <is>
+          <t>EIGHT RIVERSUITES</t>
+        </is>
+      </c>
+      <c r="P80" s="9" t="inlineStr">
+        <is>
+          <t>same location, 259:1 profitable to unprofitable</t>
+        </is>
+      </c>
       <c r="Q80" s="10" t="n"/>
     </row>
     <row r="81">
@@ -6123,8 +6451,16 @@
           <t>29c864ff55404605890dfbee32692362</t>
         </is>
       </c>
-      <c r="O85" s="9" t="n"/>
-      <c r="P85" s="9" t="n"/>
+      <c r="O85" s="9" t="inlineStr">
+        <is>
+          <t>DAIRY FARM RESIDENCES</t>
+        </is>
+      </c>
+      <c r="P85" s="9" t="inlineStr">
+        <is>
+          <t>Similar location, profitable ot unprofitable 67:3</t>
+        </is>
+      </c>
       <c r="Q85" s="10" t="n"/>
     </row>
     <row r="86">
@@ -6193,8 +6529,16 @@
           <t>23a0bd1f430c4d55a8bf6fd39fb177b8</t>
         </is>
       </c>
-      <c r="O86" s="9" t="n"/>
-      <c r="P86" s="9" t="n"/>
+      <c r="O86" s="9" t="inlineStr">
+        <is>
+          <t>GEM RESIDENCES</t>
+        </is>
+      </c>
+      <c r="P86" s="9" t="inlineStr">
+        <is>
+          <t>Close location and new, with high profitability ratio of 186:1 of profitable to unprofitable</t>
+        </is>
+      </c>
       <c r="Q86" s="10" t="n"/>
     </row>
     <row r="87">
@@ -6469,8 +6813,16 @@
           <t>70b9d30f47f5447da1d5c4252439fd26</t>
         </is>
       </c>
-      <c r="O90" s="9" t="n"/>
-      <c r="P90" s="9" t="n"/>
+      <c r="O90" s="9" t="inlineStr">
+        <is>
+          <t>THE RESERVE RESIDENCES</t>
+        </is>
+      </c>
+      <c r="P90" s="9" t="inlineStr">
+        <is>
+          <t>Similar location</t>
+        </is>
+      </c>
       <c r="Q90" s="10" t="n"/>
     </row>
     <row r="91">
@@ -6676,7 +7028,11 @@
           <t>50ba3d549264456cbe67a97565d66d79</t>
         </is>
       </c>
-      <c r="O93" s="9" t="n"/>
+      <c r="O93" s="9" t="inlineStr">
+        <is>
+          <t>JADESCAPE</t>
+        </is>
+      </c>
       <c r="P93" s="9" t="n"/>
       <c r="Q93" s="10" t="n"/>
     </row>
@@ -6745,8 +7101,16 @@
           <t>54aec0cc3a7a4a058e10fe7e21a44c17</t>
         </is>
       </c>
-      <c r="O94" s="9" t="n"/>
-      <c r="P94" s="9" t="n"/>
+      <c r="O94" s="9" t="inlineStr">
+        <is>
+          <t>ICON</t>
+        </is>
+      </c>
+      <c r="P94" s="9" t="inlineStr">
+        <is>
+          <t>Old condo (2007) but the best profitability ratio of 126:3 profitable to unprofitable in the area</t>
+        </is>
+      </c>
       <c r="Q94" s="10" t="n"/>
     </row>
     <row r="95">
@@ -6815,8 +7179,16 @@
           <t>8799614909f948d280ad127a9f14360a</t>
         </is>
       </c>
-      <c r="O95" s="9" t="n"/>
-      <c r="P95" s="9" t="n"/>
+      <c r="O95" s="9" t="inlineStr">
+        <is>
+          <t>ONE PEARL BANK</t>
+        </is>
+      </c>
+      <c r="P95" s="9" t="inlineStr">
+        <is>
+          <t>Very recent condo but profitable to unprofitable ratio is 53:11</t>
+        </is>
+      </c>
       <c r="Q95" s="10" t="n"/>
     </row>
     <row r="96">
@@ -6953,8 +7325,16 @@
           <t>cf7d4684ea39448697222b2a7d7aeab6</t>
         </is>
       </c>
-      <c r="O97" s="9" t="n"/>
-      <c r="P97" s="9" t="n"/>
+      <c r="O97" s="9" t="inlineStr">
+        <is>
+          <t>COSTA DEL SOL</t>
+        </is>
+      </c>
+      <c r="P97" s="9" t="inlineStr">
+        <is>
+          <t>Very old condo (2004) but fully profitable and same location</t>
+        </is>
+      </c>
       <c r="Q97" s="10" t="n"/>
     </row>
     <row r="98">
@@ -7298,8 +7678,16 @@
           <t>adbd4a81ec6c4032b0c6d018860067f8</t>
         </is>
       </c>
-      <c r="O102" s="9" t="n"/>
-      <c r="P102" s="9" t="n"/>
+      <c r="O102" s="9" t="inlineStr">
+        <is>
+          <t>BELLEWOODS</t>
+        </is>
+      </c>
+      <c r="P102" s="9" t="inlineStr">
+        <is>
+          <t>Similar location and both are ECs, and high profitablity ratio of 213:1 profitable to unprofitable</t>
+        </is>
+      </c>
       <c r="Q102" s="10" t="n"/>
     </row>
     <row r="103">
@@ -7367,11 +7755,18 @@
           <t>a92578afb30f481ea19b4bf48fffb96b</t>
         </is>
       </c>
-      <c r="O103" s="9" t="n"/>
-      <c r="P103" s="9" t="n"/>
+      <c r="O103" s="9" t="inlineStr">
+        <is>
+          <t>IRWELL HILL RESIDENCES</t>
+        </is>
+      </c>
+      <c r="P103" s="9" t="inlineStr">
+        <is>
+          <t>Similar location and new, good profitability ratio at 42:3 profitable to unprofitable</t>
+        </is>
+      </c>
       <c r="Q103" s="10" t="n"/>
     </row>
-    <row r="104"/>
   </sheetData>
   <autoFilter ref="A5:Q103"/>
   <mergeCells count="1">
@@ -7407,7 +7802,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -7485,7 +7879,6 @@
         <v/>
       </c>
     </row>
-    <row r="10"/>
     <row r="11">
       <c r="A11" s="11" t="inlineStr">
         <is>

</xml_diff>